<commit_message>
fixed cross-domain TPRM entity assessment import collisions during data wizard
</commit_message>
<xml_diff>
--- a/backend/data_wizard/import_templates/third_parties_template.xlsx
+++ b/backend/data_wizard/import_templates/third_parties_template.xlsx
@@ -417,24 +417,28 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -694,115 +698,115 @@
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultColWidth="8.78125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="17.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="17.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -825,78 +829,78 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.78125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="1" t="n">
         <v>3</v>
       </c>
     </row>
@@ -919,87 +923,87 @@
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="35.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="35.66"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="0" t="n">
+      <c r="F2" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="J2" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F3" s="0" t="n">
+      <c r="F3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="J3" s="0" t="s">
+      <c r="J3" s="1" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1022,157 +1026,157 @@
   <dimension ref="A1:O4"/>
   <sheetFormatPr defaultColWidth="8.78125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I2" s="0" t="n">
+      <c r="I2" s="1" t="n">
         <v>50000</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="J2" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="I3" s="0" t="n">
+      <c r="I3" s="1" t="n">
         <v>75000</v>
       </c>
-      <c r="J3" s="0" t="s">
+      <c r="J3" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="H4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I4" s="0" t="n">
+      <c r="I4" s="1" t="n">
         <v>25000</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="J4" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1195,102 +1199,102 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="63.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="21.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="63.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="21.66"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
make refid not required as we claim
</commit_message>
<xml_diff>
--- a/backend/data_wizard/import_templates/third_parties_template.xlsx
+++ b/backend/data_wizard/import_templates/third_parties_template.xlsx
@@ -84,7 +84,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="7">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -93,11 +93,8 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -108,9 +105,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -126,21 +126,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
     <cellStyle name="Currency" xfId="3" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
     <cellStyle name="Percent" xfId="5" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="6" builtinId="8"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -386,180 +385,192 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.78125" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="10" customWidth="1" style="6" min="1" max="1"/>
-    <col width="19" customWidth="1" style="6" min="2" max="2"/>
-    <col width="24" customWidth="1" style="6" min="3" max="3"/>
-    <col width="29" customWidth="1" style="6" min="4" max="4"/>
-    <col width="10" customWidth="1" style="6" min="5" max="5"/>
-    <col width="11" customWidth="1" style="6" min="6" max="6"/>
-    <col width="23" customWidth="1" style="6" min="7" max="7"/>
-    <col width="17.33" customWidth="1" style="6" min="8" max="8"/>
-    <col width="10.44" customWidth="1" style="6" min="9" max="9"/>
+    <col width="10" customWidth="1" style="7" min="1" max="1"/>
+    <col width="19" customWidth="1" style="7" min="2" max="2"/>
+    <col width="24" customWidth="1" style="7" min="3" max="3"/>
+    <col width="29" customWidth="1" style="7" min="4" max="4"/>
+    <col width="10" customWidth="1" style="7" min="5" max="5"/>
+    <col width="11" customWidth="1" style="7" min="6" max="6"/>
+    <col width="23" customWidth="1" style="7" min="7" max="7"/>
+    <col width="17.33" customWidth="1" style="7" min="8" max="8"/>
+    <col width="10.44" customWidth="1" style="7" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1" s="7">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="14.25" customHeight="1" s="8">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>ref_id</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>mission</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>country</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>parent_entity_ref_id</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>dependency</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>penetration</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>maturity</t>
         </is>
       </c>
-      <c r="K1" s="8" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>trust</t>
         </is>
       </c>
-      <c r="L1" s="8" t="inlineStr">
+      <c r="L1" s="9" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1" s="7">
-      <c r="A2" s="6" t="inlineStr">
+    <row r="2" ht="14.25" customHeight="1" s="8">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>ENT-001</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>ACME Corporation</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Cool organisation</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Provide excellent services</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1" s="7">
-      <c r="A3" s="6" t="inlineStr">
+    <row r="3" ht="14.25" customHeight="1" s="8">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>ENT-002</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>ACME Europe</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>European branch</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>European operations</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>ENT-001</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="1" s="7">
-      <c r="A4" s="6" t="inlineStr">
+    <row r="4" ht="14.25" customHeight="1" s="8">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>ENT-003</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>TechVendor Inc</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>External ICT provider</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Cloud services provider</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="14.25" customHeight="1" s="8">
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Nameless Ventures</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Newly onboarded vendor, ref_id not assigned yet</t>
         </is>
       </c>
     </row>
@@ -576,116 +587,146 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.78125" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="10" customWidth="1" style="6" min="1" max="1"/>
-    <col width="24" customWidth="1" style="6" min="2" max="2"/>
-    <col width="42" customWidth="1" style="6" min="3" max="3"/>
-    <col width="25" customWidth="1" style="6" min="4" max="4"/>
-    <col width="14" customWidth="1" style="6" min="5" max="5"/>
+    <col width="10" customWidth="1" style="7" min="1" max="1"/>
+    <col width="24" customWidth="1" style="7" min="2" max="2"/>
+    <col width="42" customWidth="1" style="7" min="3" max="3"/>
+    <col width="25" customWidth="1" style="7" min="4" max="4"/>
+    <col width="14" customWidth="1" style="7" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1" s="7">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="14.25" customHeight="1" s="8">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>ref_id</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>provider_entity_ref_id</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>criticality</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="7">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>provider_entity_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="8">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>SOL-001</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Cloud Storage Service</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Enterprise cloud storage solution</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>ENT-003</t>
         </is>
       </c>
-      <c r="E2" s="6" t="n">
+      <c r="E2" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1" s="7">
-      <c r="A3" s="6" t="inlineStr">
+    <row r="3" ht="14.25" customHeight="1" s="8">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>SOL-002</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Email Service</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Corporate email platform</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>ENT-003</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n">
+      <c r="E3" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="1" s="7">
-      <c r="A4" s="6" t="inlineStr">
+    <row r="4" ht="14.25" customHeight="1" s="8">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>SOL-003</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Internal CRM</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Customer relationship management system</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>ENT-001</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="7" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="14.25" customHeight="1" s="8">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>SOL-004</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Nameless Onboarding Service</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Pilot service from a newly onboarded vendor</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Nameless Ventures</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -704,157 +745,157 @@
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="20.22" customWidth="1" style="6" min="2" max="2"/>
-    <col width="14.09" customWidth="1" style="6" min="8" max="8"/>
-    <col width="35.66" customWidth="1" style="6" min="9" max="9"/>
-    <col width="20.59" customWidth="1" style="6" min="10" max="10"/>
+    <col width="13.11" customWidth="1" style="7" min="1" max="1"/>
+    <col width="20.22" customWidth="1" style="7" min="2" max="2"/>
+    <col width="14.09" customWidth="1" style="7" min="8" max="8"/>
+    <col width="35.66" customWidth="1" style="7" min="9" max="9"/>
+    <col width="20.59" customWidth="1" style="7" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="7">
-      <c r="A1" s="6" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="8">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>entity_ref_id</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>perimeter</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>solution_ref_id</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>criticality</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>due_date</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>audit_ref_id</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>audit_name</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="16.4" customHeight="1" s="7">
-      <c r="A2" s="6" t="inlineStr">
+    <row r="2" ht="15.75" customHeight="1" s="8">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>ENT-003</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>TechVendor Annual Security Review</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Yearly security assessment of our cloud storage provider</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>SOL-001</t>
         </is>
       </c>
-      <c r="F2" s="6" t="n">
+      <c r="F2" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>2024-12-31</t>
         </is>
       </c>
-      <c r="I2" s="9" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>ISO 27002 SOA</t>
         </is>
       </c>
-      <c r="J2" s="6" t="n"/>
-    </row>
-    <row r="3" ht="16.4" customHeight="1" s="7">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="J2" s="10" t="n"/>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" s="8">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>ENT-001</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>ACME Internal Controls Review</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Review of ACME Corporation internal controls</t>
         </is>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="F3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>2024-12-31</t>
         </is>
       </c>
-      <c r="I3" s="9" t="n"/>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="I3" s="10" t="n"/>
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>GDPR review for HR platform</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="16.4" customHeight="1" s="7">
-      <c r="A4" s="6" t="inlineStr">
+    <row r="4" ht="15.75" customHeight="1" s="8">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>ENT-002</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>ACME Controls Review</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Review of ACME Corporation internal controls</t>
         </is>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="F4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>2024-12-31</t>
         </is>
       </c>
-      <c r="I4" s="9" t="n"/>
-      <c r="J4" s="6" t="n"/>
+      <c r="I4" s="10" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -872,239 +913,239 @@
   <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.78125" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="10" customWidth="1" style="6" min="1" max="1"/>
-    <col width="25" customWidth="1" style="6" min="2" max="2"/>
-    <col width="37" customWidth="1" style="6" min="3" max="3"/>
-    <col width="25" customWidth="1" style="6" min="4" max="4"/>
-    <col width="18" customWidth="1" style="6" min="5" max="5"/>
-    <col width="9" customWidth="1" style="6" min="6" max="6"/>
-    <col width="13" customWidth="1" style="6" min="7" max="8"/>
-    <col width="17" customWidth="1" style="6" min="9" max="9"/>
-    <col width="11" customWidth="1" style="6" min="10" max="10"/>
+    <col width="10" customWidth="1" style="7" min="1" max="1"/>
+    <col width="25" customWidth="1" style="7" min="2" max="2"/>
+    <col width="37" customWidth="1" style="7" min="3" max="3"/>
+    <col width="25" customWidth="1" style="7" min="4" max="4"/>
+    <col width="18" customWidth="1" style="7" min="5" max="5"/>
+    <col width="9" customWidth="1" style="7" min="6" max="6"/>
+    <col width="13" customWidth="1" style="7" min="7" max="8"/>
+    <col width="17" customWidth="1" style="7" min="9" max="9"/>
+    <col width="11" customWidth="1" style="7" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1" s="7">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="14.25" customHeight="1" s="8">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>ref_id</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>provider_entity_ref_id</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>solution_ref_id</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>start_date</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>end_date</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>annual_expense</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="K1" s="8" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="L1" s="8" t="inlineStr">
+      <c r="L1" s="9" t="inlineStr">
         <is>
           <t>lei</t>
         </is>
       </c>
-      <c r="M1" s="8" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>euid</t>
         </is>
       </c>
-      <c r="N1" s="8" t="inlineStr">
+      <c r="N1" s="9" t="inlineStr">
         <is>
           <t>vat</t>
         </is>
       </c>
-      <c r="O1" s="8" t="inlineStr">
+      <c r="O1" s="9" t="inlineStr">
         <is>
           <t>duns</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1" s="7">
-      <c r="A2" s="6" t="inlineStr">
+    <row r="2" ht="14.25" customHeight="1" s="8">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>CON-001</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Cloud Storage Contract</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Annual cloud storage agreement</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>ENT-003</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>SOL-001</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>2024-01-01</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>2024-12-31</t>
         </is>
       </c>
-      <c r="I2" s="6" t="n">
+      <c r="I2" s="7" t="n">
         <v>50000</v>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1" s="7">
-      <c r="A3" s="6" t="inlineStr">
+    <row r="3" ht="14.25" customHeight="1" s="8">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>CON-002</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Email Services SLA</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Service level agreement for email</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>ENT-003</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>SOL-002</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>2024-01-01</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>2025-12-31</t>
         </is>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I3" s="7" t="n">
         <v>75000</v>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="1" s="7">
-      <c r="A4" s="6" t="inlineStr">
+    <row r="4" ht="14.25" customHeight="1" s="8">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>CON-003</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>CRM Maintenance</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Internal CRM maintenance agreement</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>ENT-001</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>SOL-003</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>2024-01-01</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>2024-12-31</t>
         </is>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="I4" s="7" t="n">
         <v>25000</v>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
@@ -1126,156 +1167,156 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.59765625" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="30" customWidth="1" style="6" min="1" max="1"/>
-    <col width="63.22" customWidth="1" style="6" min="4" max="4"/>
-    <col width="18.67" customWidth="1" style="6" min="5" max="5"/>
-    <col width="19" customWidth="1" style="6" min="6" max="6"/>
-    <col width="21.66" customWidth="1" style="6" min="7" max="7"/>
+    <col width="30" customWidth="1" style="7" min="1" max="1"/>
+    <col width="63.22" customWidth="1" style="7" min="4" max="4"/>
+    <col width="18.67" customWidth="1" style="7" min="5" max="5"/>
+    <col width="19" customWidth="1" style="7" min="6" max="6"/>
+    <col width="21.66" customWidth="1" style="7" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1" s="7">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="14.25" customHeight="1" s="8">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>first_name</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>last_name</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>provider_entity_ref_id</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="16.4" customHeight="1" s="7">
-      <c r="A2" s="10" t="inlineStr">
+    <row r="2" ht="15.75" customHeight="1" s="8">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>marie.durand@techvendor.com</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Marie</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>Durand</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>Main security contact for vendor communications</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>+33 1 42 00 00 01</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>CISO</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>ENT-003</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="16.4" customHeight="1" s="7">
-      <c r="A3" s="10" t="inlineStr">
+    <row r="3" ht="15.75" customHeight="1" s="8">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>thomas.leroy@acmecorp.com</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Thomas</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>Leroy</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>Administrative and contract management contact</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>+33 1 42 00 00 02</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>Compliance Manager</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="G3" s="12" t="inlineStr">
         <is>
           <t>ENT-001</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="16.4" customHeight="1" s="7">
-      <c r="A4" s="10" t="inlineStr">
+    <row r="4" ht="15.75" customHeight="1" s="8">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>alexandre.morel@acmecorp.com</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Morel</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Primary operational contact for ACME Corporation security coordination</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>+33 1 42 00 00 03</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>Security Coordinator</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="G4" s="12" t="inlineStr">
         <is>
           <t>ENT-001</t>
         </is>

</xml_diff>